<commit_message>
Added Data provider and In memory DB
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\intellij-projects\SeleniumAutomationFramework\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A45E4C-12CD-49F4-A9B0-0715EFD1E24B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B94629BB-AAD0-492F-AC9B-EC476205C916}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>sid</t>
   </si>
@@ -57,9 +57,6 @@
     <t>sid@test.com</t>
   </si>
   <si>
-    <t>Abcd@12345</t>
-  </si>
-  <si>
     <t>Chiranth</t>
   </si>
   <si>
@@ -70,6 +67,12 @@
   </si>
   <si>
     <t>Chiranth@098765</t>
+  </si>
+  <si>
+    <t>09/18/1990</t>
+  </si>
+  <si>
+    <t>SidMishra@12345</t>
   </si>
 </sst>
 </file>
@@ -114,10 +117,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -399,13 +403,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -425,7 +430,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -439,30 +444,31 @@
         <v>9</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2">
-        <v>33134</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="3"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="F3" s="2">
-        <v>33134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>